<commit_message>
Upgrade to multi-user version
</commit_message>
<xml_diff>
--- a/martins_density_map_data.xlsx
+++ b/martins_density_map_data.xlsx
@@ -8,15 +8,20 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data'!$A$1:$P$48</definedName>
+  </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.000000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,16 +37,30 @@
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7FBFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -49,14 +68,46 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D9E2F3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -462,3098 +513,3320 @@
   <dimension ref="A1:P48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.625" defaultRowHeight="15.75"/>
   <cols>
-    <col width="6.75" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="20.625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="12" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="18" bestFit="1" customWidth="1" min="2" max="2"/>
     <col width="18" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="10.25" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="40.375" customWidth="1" min="5" max="5"/>
-    <col width="19.75" customWidth="1" min="6" max="6"/>
-    <col width="11.75" customWidth="1" min="7" max="7"/>
-    <col width="10.75" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="48" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="11.375" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="10.75" bestFit="1" customWidth="1" min="11" max="11"/>
-    <col width="6.75" bestFit="1" customWidth="1" min="12" max="12"/>
-    <col width="19.875" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="14" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="42" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="13" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="13" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="10" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="18" bestFit="1" customWidth="1" min="13" max="13"/>
     <col width="18" bestFit="1" customWidth="1" min="14" max="14"/>
-    <col width="16.25" bestFit="1" customWidth="1" min="15" max="15"/>
-    <col width="14.625" bestFit="1" customWidth="1" min="16" max="16"/>
+    <col width="16" bestFit="1" customWidth="1" min="15" max="15"/>
+    <col width="16" bestFit="1" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="1" s="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="22" customFormat="1" customHeight="1" s="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>MF File</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Deceased Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Deceased Surname</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>DOD</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Province</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Full Address</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Next of Kin Name</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Next of Kin Surname</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Relationship</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Contact Number</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="4" t="n">
         <v>108364</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Zenobia </t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Haarhoff</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>31/12/2024</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>No 8 Narita Street Benoni</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Benoni</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>No 8 Narita Street Benoni, Benoni, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" s="5" t="n">
         <v>-26.1369851</v>
       </c>
-      <c r="K2" t="n">
+      <c r="K2" s="5" t="n">
         <v>27.9622093</v>
       </c>
-      <c r="L2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M2" t="inlineStr">
+      <c r="L2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Phillipus Lodewicus </t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>Haarhoff</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>Son</t>
         </is>
       </c>
-      <c r="P2" s="2" t="n">
+      <c r="P2" s="7" t="n">
         <v>832504936</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="8" t="n">
         <v>108353</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Wouter Jakobus</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Burger</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>31/12/2024</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>1241 Cornelius Street</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>Weltevredenpark</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
         <is>
           <t>1241 Cornelius Street, Weltevredenpark, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="9" t="n">
         <v>-26.1065288</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K3" s="9" t="n">
         <v>27.8113009</v>
       </c>
-      <c r="L3" t="n">
-        <v>1</v>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="L3" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Nadia Michelle </t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N3" s="8" t="inlineStr">
         <is>
           <t>Burger</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O3" s="8" t="inlineStr">
         <is>
           <t>Daughter</t>
         </is>
       </c>
-      <c r="P3" s="2" t="n">
+      <c r="P3" s="11" t="n">
         <v>737340355</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="4" t="n">
         <v>108367</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Eileen Mary</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>De Bruin</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>18/01/2025</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>J &amp; H Farming Cc R33 Belfast Carolina Road</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Belfast</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>J &amp; H Farming Cc R33 Belfast Carolina Road, Belfast, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="J4" t="n">
+      <c r="J4" s="5" t="n">
         <v>-26.1068543</v>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" s="5" t="n">
         <v>27.810501</v>
       </c>
-      <c r="L4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M4" t="inlineStr">
+      <c r="L4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Carol De </t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>Bruin</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>Daughter In Law</t>
         </is>
       </c>
-      <c r="P4" s="2" t="n">
+      <c r="P4" s="7" t="n">
         <v>824470601</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="8" t="n">
         <v>108342</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Zelton </t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Wisken</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>24/01/2025</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Emily Hob House Street </t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>Johannesburg</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>Emily Hob House Street, Johannesburg, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="9" t="n">
         <v>-26.1061416</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" s="9" t="n">
         <v>27.8108691</v>
       </c>
-      <c r="L5" t="n">
-        <v>1</v>
-      </c>
-      <c r="M5" t="inlineStr">
+      <c r="L5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>candice Burnett</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N5" s="8" t="inlineStr">
         <is>
           <t>Olivier</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O5" s="8" t="inlineStr">
         <is>
           <t>Daughter</t>
         </is>
       </c>
-      <c r="P5" s="2" t="n">
+      <c r="P5" s="11" t="n">
         <v>837257173</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="4" t="n">
         <v>108337</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Janice Ann</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Summers Swanepoel</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>18/01/2025</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>13 Dyeri Place , Florida Glen</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Florida Glen</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>13 Dyeri Place , Florida Glen, Florida Glen, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="J6" t="n">
+      <c r="J6" s="5" t="n">
         <v>-26.1070233</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K6" s="5" t="n">
         <v>27.8119779</v>
       </c>
-      <c r="L6" t="n">
-        <v>1</v>
-      </c>
-      <c r="M6" t="inlineStr">
+      <c r="L6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Martin </t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>Swanepoel</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>Son</t>
         </is>
       </c>
-      <c r="P6" s="2" t="n">
+      <c r="P6" s="7" t="n">
         <v>716713301</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="8" t="n">
         <v>108340</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Nkanyiso</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Mpofu</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>22/01/2025</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>26 Knoppiesdoring Rd</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Randpark Ridge</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>26 Knoppiesdoring Rd, Randpark Ridge, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="J7" s="9" t="n"/>
+      <c r="K7" s="9" t="n"/>
+      <c r="L7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Thandi </t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N7" s="8" t="inlineStr">
         <is>
           <t>Mpofu</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O7" s="8" t="inlineStr">
         <is>
           <t>Daughter</t>
         </is>
       </c>
-      <c r="P7" s="2" t="n">
+      <c r="P7" s="11" t="n">
         <v>616548663</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="4" t="n">
         <v>108341</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Fikile Sheila </t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Danisa</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>23/01/2025</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>109 Area Road Judiths Bethrams</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Johannesburg</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>109 Area Road Judiths Bethrams, Johannesburg, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="J8" s="5" t="n"/>
+      <c r="K8" s="5" t="n"/>
+      <c r="L8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Lindokuhle Pretty </t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N8" s="4" t="inlineStr">
         <is>
           <t>Nkosi</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="O8" s="4" t="inlineStr">
         <is>
           <t>Sister</t>
         </is>
       </c>
-      <c r="P8" s="2" t="n">
+      <c r="P8" s="7" t="n">
         <v>844151093</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="8" t="n">
         <v>108334</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Kenneth Norman</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Hewson</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>14/01/2025</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>73 Nelson Street</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Northcliff</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
         <is>
           <t>73 Nelson Street, Northcliff, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="J9" s="9" t="n"/>
+      <c r="K9" s="9" t="n"/>
+      <c r="L9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Colleen </t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N9" s="8" t="inlineStr">
         <is>
           <t>Brookes</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="O9" s="8" t="inlineStr">
         <is>
           <t>Daughter</t>
         </is>
       </c>
-      <c r="P9" s="2" t="n">
+      <c r="P9" s="11" t="n">
         <v>768504731</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="4" t="n">
         <v>108339</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Liam </t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Olivier</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>20/01/2025</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>Unit 50 San Marco Estate Kelly Avenue, Bromhof</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>Randburg</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Unit 50 San Marco Estate Kelly Avenue, Bromhof, Randburg, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="J10" s="5" t="n"/>
+      <c r="K10" s="5" t="n"/>
+      <c r="L10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Emily-Kate </t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>Olivier</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>Mother</t>
         </is>
       </c>
-      <c r="P10" s="2" t="n">
+      <c r="P10" s="7" t="n">
         <v>829773846</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="8" t="n">
         <v>108316</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Michael Detroid</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Van Tonder</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>23/12/2024</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>203, st Amant Street Malvern</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>Johannesburg</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
         <is>
           <t>203, st Amant Street Malvern, Johannesburg, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="9" t="n"/>
+      <c r="L11" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Dawn Elizabeth </t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="N11" s="8" t="inlineStr">
         <is>
           <t>Jacobs</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="O11" s="8" t="inlineStr">
         <is>
           <t>Common Law Wife</t>
         </is>
       </c>
-      <c r="P11" s="2" t="n">
+      <c r="P11" s="11" t="n">
         <v>643664928</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="4" t="n">
         <v>108345</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Cornelia Elzabe</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Malan</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>02/02/2025</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>89 Marigould Str Benoni</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>Johannesburg</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>89 Marigould Str Benoni, Johannesburg, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="J12" s="5" t="n"/>
+      <c r="K12" s="5" t="n"/>
+      <c r="L12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Daniel Jacobus Roeloff </t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="N12" s="4" t="inlineStr">
         <is>
           <t>Malan</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="O12" s="4" t="inlineStr">
         <is>
           <t>Husband</t>
         </is>
       </c>
-      <c r="P12" s="2" t="n">
+      <c r="P12" s="7" t="n">
         <v>685670919</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="8" t="n">
         <v>108343</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Ricardo </t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Coetzee</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>03/02/2025</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>200 Uys Street, Rynveld</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>Benoni</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
         <is>
           <t>200 Uys Street, Rynveld, Benoni, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="J13" s="9" t="n"/>
+      <c r="K13" s="9" t="n"/>
+      <c r="L13" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Ruan </t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="N13" s="8" t="inlineStr">
         <is>
           <t>Coetzee</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="O13" s="8" t="inlineStr">
         <is>
           <t>Father</t>
         </is>
       </c>
-      <c r="P13" s="2" t="n">
+      <c r="P13" s="11" t="n">
         <v>766153142</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="4" t="n">
         <v>108398</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Veuna Ilona</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Custers</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>16/02/2025</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">17 Huilboom Street </t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>Randpark Ridge</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>17 Huilboom Street, Randpark Ridge, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="J14" s="5" t="n"/>
+      <c r="K14" s="5" t="n"/>
+      <c r="L14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Jennifer </t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t>Custers</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="O14" s="4" t="inlineStr">
         <is>
           <t>Daughter</t>
         </is>
       </c>
-      <c r="P14" s="2" t="n">
+      <c r="P14" s="7" t="n">
         <v>828289824</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="8" t="n">
         <v>108348</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Louise Kathleen</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Wijtenburg</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>15/02/2025</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>10 A 8th Avenue Parktown North</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>Parktown</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
         <is>
           <t>10 A 8th Avenue Parktown North, Parktown, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="J15" s="9" t="n"/>
+      <c r="K15" s="9" t="n"/>
+      <c r="L15" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Mark </t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="N15" s="8" t="inlineStr">
         <is>
           <t>Wijtenburg</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="O15" s="8" t="inlineStr">
         <is>
           <t>Son</t>
         </is>
       </c>
-      <c r="P15" s="2" t="n">
+      <c r="P15" s="11" t="n">
         <v>834099942</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="4" t="n">
         <v>108397</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Henry Andrew</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Truter</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>17/02/2025</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>5 Rivonia Village, Whelan Close, Sandton</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Sandton Johannesburg</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>5 Rivonia Village, Whelan Close, Sandton, Sandton Johannesburg, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="J16" s="5" t="n"/>
+      <c r="K16" s="5" t="n"/>
+      <c r="L16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Shelley Dianne </t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="N16" s="4" t="inlineStr">
         <is>
           <t>Truter</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="O16" s="4" t="inlineStr">
         <is>
           <t>Wife</t>
         </is>
       </c>
-      <c r="P16" s="2" t="n">
+      <c r="P16" s="7" t="n">
         <v>824023728</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="8" t="n">
         <v>108349</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Ryan Simon</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>Ottens</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>24/02/2025</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Unit 7 , 17 on Forest Drive, Lonehill</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>Lonehill  Johannesburg</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
         <is>
           <t>Unit 7 , 17 on Forest Drive, Lonehill, Lonehill  Johannesburg, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="J17" s="9" t="n"/>
+      <c r="K17" s="9" t="n"/>
+      <c r="L17" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Chanti-lez </t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="N17" s="8" t="inlineStr">
         <is>
           <t>Ottens</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="O17" s="8" t="inlineStr">
         <is>
           <t>Wife</t>
         </is>
       </c>
-      <c r="P17" s="2" t="n">
+      <c r="P17" s="11" t="n">
         <v>825340916</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="4" t="n">
         <v>108381</v>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Coral Diane</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Kerr</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>24/02/2025</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>31 Thornfields Estate 18 Rye Lane Magaliessig Sandton</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>Sandton Johannesburg</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>31 Thornfields Estate 18 Rye Lane Magaliessig Sandton, Sandton Johannesburg, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="J18" s="5" t="n"/>
+      <c r="K18" s="5" t="n"/>
+      <c r="L18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Linda </t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="N18" s="4" t="inlineStr">
         <is>
           <t>Von Holdt</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="O18" s="4" t="inlineStr">
         <is>
           <t>Sister</t>
         </is>
       </c>
-      <c r="P18" s="2" t="n">
+      <c r="P18" s="7" t="n">
         <v>833361505</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" s="8" t="n">
         <v>108361</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Therese Erna Mary</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Smit</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>24/02/2025</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>13 Juniper Street</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>Randpark Ridge</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
         <is>
           <t>13 Juniper Street, Randpark Ridge, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="J19" s="9" t="n"/>
+      <c r="K19" s="9" t="n"/>
+      <c r="L19" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Frederick Rick </t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="N19" s="8" t="inlineStr">
         <is>
           <t>Smit</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="O19" s="8" t="inlineStr">
         <is>
           <t>Son</t>
         </is>
       </c>
-      <c r="P19" s="2" t="n">
+      <c r="P19" s="11" t="n">
         <v>832962391</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="4" t="n">
         <v>108368</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Edward Albert </t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Newton</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>22/02/2025</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">166 Mowbray Road </t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>Greenside</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>166 Mowbray Road, Greenside, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="J20" s="5" t="n"/>
+      <c r="K20" s="5" t="n"/>
+      <c r="L20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Alison Douglas </t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="N20" s="4" t="inlineStr">
         <is>
           <t>Newton</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="O20" s="4" t="inlineStr">
         <is>
           <t>Wife</t>
         </is>
       </c>
-      <c r="P20" s="2" t="n">
+      <c r="P20" s="7" t="n">
         <v>768913831</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="8" t="n">
         <v>108369</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>Anthony John</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Walker</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>23/02/2025</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>Unit 4385 Waterfall Midrand</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>Kyalami</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Unit 4385 Waterfall Midrand, Kyalami, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="J21" s="9" t="n"/>
+      <c r="K21" s="9" t="n"/>
+      <c r="L21" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Scott Anthony </t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="N21" s="8" t="inlineStr">
         <is>
           <t>Walker</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="O21" s="8" t="inlineStr">
         <is>
           <t>Son</t>
         </is>
       </c>
-      <c r="P21" s="2" t="n">
+      <c r="P21" s="11" t="n">
         <v>795160399</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" s="4" t="n">
         <v>108344</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>James Brain</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Bowes</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>01/02/2025</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>Landseer Close, Wellingboraish</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>England</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>UK</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>Landseer Close, Wellingboraish, England, UK, South Africa</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="J22" s="5" t="n"/>
+      <c r="K22" s="5" t="n"/>
+      <c r="L22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Karen Ann </t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="N22" s="4" t="inlineStr">
         <is>
           <t>Bowes</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="O22" s="4" t="inlineStr">
         <is>
           <t>Daughter</t>
         </is>
       </c>
-      <c r="P22" s="2" t="n">
+      <c r="P22" s="7" t="n">
         <v>833009175</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" s="8" t="n">
         <v>108360</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>Pamela Wendy</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Turner</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>23/02/2025</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>63 Imbuia Street Northcliff</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>Northcliff</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
         <is>
           <t>63 Imbuia Street Northcliff, Northcliff, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="J23" s="9" t="n"/>
+      <c r="K23" s="9" t="n"/>
+      <c r="L23" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M23" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Eloise Julia Clarke </t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="N23" s="8" t="inlineStr">
         <is>
           <t>Lewis - Enright</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="O23" s="8" t="inlineStr">
         <is>
           <t>Daughter</t>
         </is>
       </c>
-      <c r="P23" s="2" t="n">
+      <c r="P23" s="11" t="n">
         <v>833819083</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
+      <c r="A24" s="4" t="n">
         <v>108380</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Avril Mary</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Langley</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>26/02/2025</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>2 Aleit Road,  Aldara Park</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>Randburg</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>2 Aleit Road,  Aldara Park, Randburg, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="J24" s="5" t="n"/>
+      <c r="K24" s="5" t="n"/>
+      <c r="L24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Cynthia Gay </t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="N24" s="4" t="inlineStr">
         <is>
           <t>Alexander</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="O24" s="4" t="inlineStr">
         <is>
           <t>Friend</t>
         </is>
       </c>
-      <c r="P24" s="2" t="n">
+      <c r="P24" s="7" t="n">
         <v>824628990</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
+      <c r="A25" s="8" t="n">
         <v>108347</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>Petronella Margaretha</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>Dege</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>09/02/2025</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>8 Ebony Drive, Northcliff</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>Northcliff</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
         <is>
           <t>8 Ebony Drive, Northcliff, Northcliff, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="J25" s="9" t="n"/>
+      <c r="K25" s="9" t="n"/>
+      <c r="L25" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M25" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Rone - Marie </t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="N25" s="8" t="inlineStr">
         <is>
           <t>Keet</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
+      <c r="O25" s="8" t="inlineStr">
         <is>
           <t>Daughter</t>
         </is>
       </c>
-      <c r="P25" s="2" t="n">
+      <c r="P25" s="11" t="n">
         <v>620652849</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
+      <c r="A26" s="4" t="n">
         <v>108330</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Florence Theresa Tuohy</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Fenn</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>31/01/2025</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>20 Musilis Drive</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>Northcliff</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
         <is>
           <t>20 Musilis Drive, Northcliff, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="J26" s="5" t="n"/>
+      <c r="K26" s="5" t="n"/>
+      <c r="L26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Terrence Kevin </t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="N26" s="4" t="inlineStr">
         <is>
           <t>Fenn</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
+      <c r="O26" s="4" t="inlineStr">
         <is>
           <t>Son</t>
         </is>
       </c>
-      <c r="P26" s="2" t="n">
+      <c r="P26" s="7" t="n">
         <v>835563453</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="n">
+      <c r="A27" s="8" t="n">
         <v>108419</v>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>Cynthia Ann</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>Reuvers</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>26/03/2025</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>1237 Cornelius Street , 39 Oakfield Place</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>Weltevredenpark</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
         <is>
           <t>1237 Cornelius Street , 39 Oakfield Place, Weltevredenpark, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="J27" s="9" t="n"/>
+      <c r="K27" s="9" t="n"/>
+      <c r="L27" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M27" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Charles </t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="N27" s="8" t="inlineStr">
         <is>
           <t>Reuvers</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="O27" s="8" t="inlineStr">
         <is>
           <t>Son</t>
         </is>
       </c>
-      <c r="P27" s="2" t="n">
+      <c r="P27" s="11" t="n">
         <v>842892712</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
+      <c r="A28" s="4" t="n">
         <v>108411</v>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Beryl Hazel</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Higgins</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>29/03/2025</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>21 Senior Drive, Blackheath, Northcliff</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>Northcliff</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>21 Senior Drive, Blackheath, Northcliff, Northcliff, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="J28" s="5" t="n"/>
+      <c r="K28" s="5" t="n"/>
+      <c r="L28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M28" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Gillian Diane </t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="N28" s="4" t="inlineStr">
         <is>
           <t>Higgins</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
+      <c r="O28" s="4" t="inlineStr">
         <is>
           <t>Daughter</t>
         </is>
       </c>
-      <c r="P28" s="2" t="n">
+      <c r="P28" s="7" t="n">
         <v>813812668</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="8" t="n">
         <v>108373</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>Irma</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>Du Plessis</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="8" t="inlineStr">
         <is>
           <t>01/03/2025</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="8" t="inlineStr">
         <is>
           <t>24 Villa Rade, Nusery Close Westering</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F29" s="8" t="inlineStr">
         <is>
           <t>Westering</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="8" t="inlineStr">
         <is>
           <t>Eastern Cape</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
         <is>
           <t>24 Villa Rade, Nusery Close Westering, Westering, Eastern Cape, South Africa</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="J29" s="9" t="n"/>
+      <c r="K29" s="9" t="n"/>
+      <c r="L29" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M29" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Gerhardus Petrus </t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="N29" s="8" t="inlineStr">
         <is>
           <t>Van Rhyn</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="O29" s="8" t="inlineStr">
         <is>
           <t>Son Inlaw</t>
         </is>
       </c>
-      <c r="P29" s="2" t="n">
+      <c r="P29" s="11" t="n">
         <v>722468001</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="n">
+      <c r="A30" s="4" t="n">
         <v>108375</v>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>John Spencer</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Mcgowan</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>08/03/2025</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>229 Arkansas Avenue Berario</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>Berario</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>229 Arkansas Avenue Berario, Berario, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="J30" s="5" t="n"/>
+      <c r="K30" s="5" t="n"/>
+      <c r="L30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M30" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Robert Michael </t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="N30" s="4" t="inlineStr">
         <is>
           <t>Mcgowan</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
+      <c r="O30" s="4" t="inlineStr">
         <is>
           <t>Son</t>
         </is>
       </c>
-      <c r="P30" s="2" t="n">
+      <c r="P30" s="7" t="n">
         <v>836018511</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="8" t="n">
         <v>108377</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>Johannes Cornelis</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>Kotze</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>14/03/2025</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
         <is>
           <t>176 Senior Drive Northcliff</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="8" t="inlineStr">
         <is>
           <t>Northcliff</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H31" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
         <is>
           <t>176 Senior Drive Northcliff, Northcliff, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="J31" s="9" t="n"/>
+      <c r="K31" s="9" t="n"/>
+      <c r="L31" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M31" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Christelle Mimi </t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="N31" s="8" t="inlineStr">
         <is>
           <t>Kotze</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
+      <c r="O31" s="8" t="inlineStr">
         <is>
           <t>Wife</t>
         </is>
       </c>
-      <c r="P31" s="2" t="n">
+      <c r="P31" s="11" t="n">
         <v>820622090</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="n">
+      <c r="A32" s="4" t="n">
         <v>108359</v>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>Daniel Rossouw Burger</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>Hanekom</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>02/03/2025</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
         <is>
           <t>1 Nolene Street, Constantia Kloof</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>Roodepoort</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
         <is>
           <t>1 Nolene Street, Constantia Kloof, Roodepoort, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="J32" s="5" t="n"/>
+      <c r="K32" s="5" t="n"/>
+      <c r="L32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Lorinda Johanna </t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="N32" s="4" t="inlineStr">
         <is>
           <t>Hanekom</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
+      <c r="O32" s="4" t="inlineStr">
         <is>
           <t>Wife</t>
         </is>
       </c>
-      <c r="P32" s="2" t="n">
+      <c r="P32" s="7" t="n">
         <v>824479086</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="n">
+      <c r="A33" s="8" t="n">
         <v>108414</v>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>Shirley Rose</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>Hurley</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="8" t="inlineStr">
         <is>
           <t>19/03/2025</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="8" t="inlineStr">
         <is>
           <t>721 Shelter Avenue, Little Falls</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="8" t="inlineStr">
         <is>
           <t>Roodepoort</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
         <is>
           <t>721 Shelter Avenue, Little Falls, Roodepoort, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="J33" s="9" t="n"/>
+      <c r="K33" s="9" t="n"/>
+      <c r="L33" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M33" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Cheryl Loreen </t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
+      <c r="N33" s="8" t="inlineStr">
         <is>
           <t>Howes</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr">
+      <c r="O33" s="8" t="inlineStr">
         <is>
           <t>Daughter</t>
         </is>
       </c>
-      <c r="P33" s="2" t="n">
+      <c r="P33" s="11" t="n">
         <v>726416669</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
+      <c r="A34" s="4" t="n">
         <v>108415</v>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>Norman Maurice Carew</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>Hodge</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>24/03/2025</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
         <is>
           <t>9 Virgo Avenue Sundowner</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>Sundowner</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
         <is>
           <t>9 Virgo Avenue Sundowner, Sundowner, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="J34" s="5" t="n"/>
+      <c r="K34" s="5" t="n"/>
+      <c r="L34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M34" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Ryan </t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="N34" s="4" t="inlineStr">
         <is>
           <t>Hodge</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr">
+      <c r="O34" s="4" t="inlineStr">
         <is>
           <t>Son</t>
         </is>
       </c>
-      <c r="P34" s="2" t="n">
+      <c r="P34" s="7" t="n">
         <v>828757294</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="n">
+      <c r="A35" s="8" t="n">
         <v>108356</v>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>Amanda</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
         <is>
           <t>Clark</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="8" t="inlineStr">
         <is>
           <t>26/03/2025</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="8" t="inlineStr">
         <is>
           <t>12 Annie Street Fontainebleau</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="8" t="inlineStr">
         <is>
           <t>Randburg</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
         <is>
           <t>12 Annie Street Fontainebleau, Randburg, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="J35" s="9" t="n"/>
+      <c r="K35" s="9" t="n"/>
+      <c r="L35" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M35" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Chantelle </t>
         </is>
       </c>
-      <c r="N35" t="inlineStr">
+      <c r="N35" s="8" t="inlineStr">
         <is>
           <t>Clark</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
+      <c r="O35" s="8" t="inlineStr">
         <is>
           <t>Daughter</t>
         </is>
       </c>
-      <c r="P35" s="2" t="n">
+      <c r="P35" s="11" t="n">
         <v>640041373</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="n">
+      <c r="A36" s="4" t="n">
         <v>108418</v>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>Stanley Arthur</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Lindsay</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>26/03/2025</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Unit 6 Nelinda Hills </t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>Wilgerheuwel</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
         <is>
           <t>Unit 6 Nelinda Hills, Wilgerheuwel, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="J36" s="5" t="n"/>
+      <c r="K36" s="5" t="n"/>
+      <c r="L36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M36" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Susan Alexana </t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
+      <c r="N36" s="4" t="inlineStr">
         <is>
           <t>Lindsay</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
+      <c r="O36" s="4" t="inlineStr">
         <is>
           <t>Wife</t>
         </is>
       </c>
-      <c r="P36" s="2" t="n">
+      <c r="P36" s="7" t="n">
         <v>823004123</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="n">
+      <c r="A37" s="8" t="n">
         <v>108413</v>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>Roy Anthony</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>Brentnall</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="8" t="inlineStr">
         <is>
           <t>27/03/2025</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="8" t="inlineStr">
         <is>
           <t>1 Kessel Close, 175 Kessel Street Fairland</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="8" t="inlineStr">
         <is>
           <t>Fairland</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
         <is>
           <t>1 Kessel Close, 175 Kessel Street Fairland, Fairland, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="J37" s="9" t="n"/>
+      <c r="K37" s="9" t="n"/>
+      <c r="L37" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M37" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Charmaine Monica </t>
         </is>
       </c>
-      <c r="N37" t="inlineStr">
+      <c r="N37" s="8" t="inlineStr">
         <is>
           <t>Brentnall</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr">
+      <c r="O37" s="8" t="inlineStr">
         <is>
           <t>Daughter</t>
         </is>
       </c>
-      <c r="P37" s="2" t="n">
+      <c r="P37" s="11" t="n">
         <v>833071104</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="n">
+      <c r="A38" s="4" t="n">
         <v>108412</v>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>Beatrix Gezina</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>Wood</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>25/03/2025</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="4" t="inlineStr">
         <is>
           <t>7 Fortune Gate Weltevredenpark</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="4" t="inlineStr">
         <is>
           <t>Weltevredenpark</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
         <is>
           <t>7 Fortune Gate Weltevredenpark, Weltevredenpark, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="J38" s="5" t="n"/>
+      <c r="K38" s="5" t="n"/>
+      <c r="L38" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M38" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Lea </t>
         </is>
       </c>
-      <c r="N38" t="inlineStr">
+      <c r="N38" s="4" t="inlineStr">
         <is>
           <t>Kreutzfeldt</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr">
+      <c r="O38" s="4" t="inlineStr">
         <is>
           <t>Sister</t>
         </is>
       </c>
-      <c r="P38" s="2" t="n">
+      <c r="P38" s="7" t="n">
         <v>834080880</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="8" t="n">
         <v>108378</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>John Graham</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="8" t="inlineStr">
         <is>
           <t>Hunter</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="8" t="inlineStr">
         <is>
           <t>17/03/2025</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="8" t="inlineStr">
         <is>
           <t>21 Talbrager Avenue</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="8" t="inlineStr">
         <is>
           <t>Graighall</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H39" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
         <is>
           <t>21 Talbrager Avenue, Graighall, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="J39" s="9" t="n"/>
+      <c r="K39" s="9" t="n"/>
+      <c r="L39" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M39" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Joan Leslie </t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
+      <c r="N39" s="8" t="inlineStr">
         <is>
           <t>Hunter</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr">
+      <c r="O39" s="8" t="inlineStr">
         <is>
           <t>Wife</t>
         </is>
       </c>
-      <c r="P39" s="2" t="n">
+      <c r="P39" s="11" t="n">
         <v>794696830</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
+      <c r="A40" s="4" t="n">
         <v>108379</v>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>Ian</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>Cloete</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>17/03/2025</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>9 Wilde Amandel Street</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr">
         <is>
           <t>Ferndale</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
         <is>
           <t>9 Wilde Amandel Street, Ferndale, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="J40" s="5" t="n"/>
+      <c r="K40" s="5" t="n"/>
+      <c r="L40" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M40" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Stella </t>
         </is>
       </c>
-      <c r="N40" t="inlineStr">
+      <c r="N40" s="4" t="inlineStr">
         <is>
           <t>Cloete</t>
         </is>
       </c>
-      <c r="P40" s="2" t="n">
+      <c r="O40" s="4" t="n"/>
+      <c r="P40" s="7" t="n">
         <v>790907771</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="n">
+      <c r="A41" s="8" t="n">
         <v>108374</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="8" t="inlineStr">
         <is>
           <t>Gabriella Wyhona</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="8" t="inlineStr">
         <is>
           <t>Pillay</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="8" t="inlineStr">
         <is>
           <t>06/03/2025</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="8" t="inlineStr">
         <is>
           <t>102 Zeiss Road, Eagles Reef, Honeydew</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="8" t="inlineStr">
         <is>
           <t>Honeydew</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="inlineStr">
         <is>
           <t>102 Zeiss Road, Eagles Reef, Honeydew, Honeydew, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="J41" s="9" t="n"/>
+      <c r="K41" s="9" t="n"/>
+      <c r="L41" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M41" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Jadine Brittany </t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
+      <c r="N41" s="8" t="inlineStr">
         <is>
           <t>Narayanasami</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr">
+      <c r="O41" s="8" t="inlineStr">
         <is>
           <t>Mother</t>
         </is>
       </c>
-      <c r="P41" s="2" t="n">
+      <c r="P41" s="11" t="n">
         <v>714416603</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="n">
+      <c r="A42" s="4" t="n">
         <v>108376</v>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Jean Glenville </t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>Magnus</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr">
         <is>
           <t>11/03/2025</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="4" t="inlineStr">
         <is>
           <t>159 A Acacia Road Northcliff</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="4" t="inlineStr">
         <is>
           <t>Northcliff</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I42" s="4" t="inlineStr">
         <is>
           <t>159 A Acacia Road Northcliff, Northcliff, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="J42" s="5" t="n"/>
+      <c r="K42" s="5" t="n"/>
+      <c r="L42" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M42" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Lara </t>
         </is>
       </c>
-      <c r="N42" t="inlineStr">
+      <c r="N42" s="4" t="inlineStr">
         <is>
           <t>Magnus - Mcarthur</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr">
+      <c r="O42" s="4" t="inlineStr">
         <is>
           <t>Daughter</t>
         </is>
       </c>
-      <c r="P42" s="2" t="n">
+      <c r="P42" s="7" t="n">
         <v>829258602</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="8" t="n">
         <v>108382</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Paul Jacobus </t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="8" t="inlineStr">
         <is>
           <t>Wessels</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="8" t="inlineStr">
         <is>
           <t>03/03/2025</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" s="8" t="inlineStr">
         <is>
           <t>5 Eloff Street Crystal Park</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="8" t="inlineStr">
         <is>
           <t>Crystal Park</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="inlineStr">
         <is>
           <t>5 Eloff Street Crystal Park, Crystal Park, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="J43" s="9" t="n"/>
+      <c r="K43" s="9" t="n"/>
+      <c r="L43" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M43" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Ingrid Tienie </t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
+      <c r="N43" s="8" t="inlineStr">
         <is>
           <t>Wessels</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr">
+      <c r="O43" s="8" t="inlineStr">
         <is>
           <t>Wife</t>
         </is>
       </c>
-      <c r="P43" s="2" t="n">
+      <c r="P43" s="11" t="n">
         <v>728412302</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="n">
+      <c r="A44" s="4" t="n">
         <v>108417</v>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>Gregory Charles</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>Farnworth</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>24/03/2025</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E44" s="4" t="inlineStr">
         <is>
           <t>23 St Martin Cocoa Close Honeydew</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>Honeydew</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
         <is>
           <t>23 St Martin Cocoa Close Honeydew, Honeydew, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr">
+      <c r="J44" s="5" t="n"/>
+      <c r="K44" s="5" t="n"/>
+      <c r="L44" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M44" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Paul </t>
         </is>
       </c>
-      <c r="N44" t="inlineStr">
+      <c r="N44" s="4" t="inlineStr">
         <is>
           <t>Farnworth</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr">
+      <c r="O44" s="4" t="inlineStr">
         <is>
           <t>Son</t>
         </is>
       </c>
-      <c r="P44" s="2" t="n">
+      <c r="P44" s="7" t="n">
         <v>834693190</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="8" t="n">
         <v>108416</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="8" t="inlineStr">
         <is>
           <t>Evelyn Joan</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="8" t="inlineStr">
         <is>
           <t>Tinkler</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="8" t="inlineStr">
         <is>
           <t>24/03/2025</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="8" t="inlineStr">
         <is>
           <t>10 Wattle Street Northmead ext 4</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="8" t="inlineStr">
         <is>
           <t>Benoni</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H45" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I45" s="8" t="inlineStr">
         <is>
           <t>10 Wattle Street Northmead ext 4, Benoni, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="J45" s="9" t="n"/>
+      <c r="K45" s="9" t="n"/>
+      <c r="L45" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M45" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">David Noel </t>
         </is>
       </c>
-      <c r="N45" t="inlineStr">
+      <c r="N45" s="8" t="inlineStr">
         <is>
           <t>Tinkler</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr">
+      <c r="O45" s="8" t="inlineStr">
         <is>
           <t>Son</t>
         </is>
       </c>
-      <c r="P45" s="2" t="n">
+      <c r="P45" s="11" t="n">
         <v>829493565</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
+      <c r="A46" s="4" t="n">
         <v>108420</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>Karel Frederik</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>Cornelius</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>26/03/2025</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>11 Roodeberg, Garrick Street Rangview</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="4" t="inlineStr">
         <is>
           <t>Krugersdorp</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
         <is>
           <t>11 Roodeberg, Garrick Street Rangview, Krugersdorp, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
+      <c r="J46" s="5" t="n"/>
+      <c r="K46" s="5" t="n"/>
+      <c r="L46" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M46" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Isabella Maria </t>
         </is>
       </c>
-      <c r="N46" t="inlineStr">
+      <c r="N46" s="4" t="inlineStr">
         <is>
           <t>Cornelius</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr">
+      <c r="O46" s="4" t="inlineStr">
         <is>
           <t>Daughter</t>
         </is>
       </c>
-      <c r="P46" s="2" t="n">
+      <c r="P46" s="7" t="n">
         <v>834734896</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="n">
+      <c r="A47" s="8" t="n">
         <v>108396</v>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="8" t="inlineStr">
         <is>
           <t>Brian Ellis</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="8" t="inlineStr">
         <is>
           <t>Parry</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="8" t="inlineStr">
         <is>
           <t>28/03/2025</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E47" s="8" t="inlineStr">
         <is>
           <t>25 Signal Avenue, Dawnview,</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="8" t="inlineStr">
         <is>
           <t>Germiston</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Gauteng</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>Gauteng</t>
+        </is>
+      </c>
+      <c r="H47" s="8" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I47" s="8" t="inlineStr">
         <is>
           <t>25 Signal Avenue, Dawnview,, Germiston, Gauteng, South Africa</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr">
+      <c r="J47" s="9" t="n"/>
+      <c r="K47" s="9" t="n"/>
+      <c r="L47" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M47" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Lynette </t>
         </is>
       </c>
-      <c r="N47" t="inlineStr">
+      <c r="N47" s="8" t="inlineStr">
         <is>
           <t>Parry</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr">
+      <c r="O47" s="8" t="inlineStr">
         <is>
           <t>Wife</t>
         </is>
       </c>
-      <c r="P47" s="2" t="n">
+      <c r="P47" s="11" t="n">
         <v>614924903</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="n">
+      <c r="A48" s="4" t="n">
         <v>108384</v>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>Cheryl Anne Marguerite</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>Vd Westhuizen</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="4" t="inlineStr">
         <is>
           <t>30/03/2025</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E48" s="4" t="inlineStr">
         <is>
           <t>143 17th Street E , North Vancouver</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="4" t="inlineStr">
         <is>
           <t>North Vancouver</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="G48" s="4" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="I48" s="4" t="inlineStr">
         <is>
           <t>143 17th Street E , North Vancouver, North Vancouver, Canada, South Africa</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
+      <c r="J48" s="5" t="n"/>
+      <c r="K48" s="5" t="n"/>
+      <c r="L48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M48" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Richard </t>
         </is>
       </c>
-      <c r="N48" t="inlineStr">
+      <c r="N48" s="4" t="inlineStr">
         <is>
           <t>Vd Westhuizen</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr">
+      <c r="O48" s="4" t="inlineStr">
         <is>
           <t>Son</t>
         </is>
       </c>
-      <c r="P48" s="2" t="n">
+      <c r="P48" s="7" t="n">
         <v>835060092</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:P48"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>